<commit_message>
feat: add confirmation attendance script and update menu options
</commit_message>
<xml_diff>
--- a/dataset/pelayanan_sekolah.xlsx
+++ b/dataset/pelayanan_sekolah.xlsx
@@ -567,7 +567,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:DA4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" outlineLevelCol="0"/>
   <cols>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
     <col width="12.6640625" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
@@ -1195,17 +1195,17 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>Kelas 1</t>
+          <t>Kelas 2</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>junior</t>
+          <t>Putri Shidqiyah</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>FAILED: None of the expected buttons appeared</t>
+          <t>FAILED: 'nama_lengkap'</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">

</xml_diff>